<commit_message>
Update: push latest changes
</commit_message>
<xml_diff>
--- a/reports/test_execution_report.xlsx
+++ b/reports/test_execution_report.xlsx
@@ -487,7 +487,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-13T11:45:00</t>
+          <t>2026-06-13T14:31:15</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,40 +513,55 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Step Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Step Status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Step Message</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>From</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Journey Type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Duration (s)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Screenshot</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
@@ -560,118 +575,895 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Search flights using Cleartrip flow</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Flight search completed for Mumbai to Delhi</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Delhi</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>One Way</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>18.03</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=20/06/2026&amp;from=BOM&amp;to=DEL&amp;intl=n&amp;origin=BOM%20-%20Mumbai,%20IN&amp;destination=DEL%20-%20New%20Delhi,%20IN&amp;sft=&amp;sd=1781331259373&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-06-13T11:44:30</t>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=20/06/2026&amp;from=BOM&amp;to=DEL&amp;intl=n&amp;origin=BOM%20-%20Mumbai,%20IN&amp;destination=DEL%20-%20New%20Delhi,%20IN&amp;sft=&amp;sd=1781341242090&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC001.png</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:30:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TC002</t>
+          <t>TC001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Validate airline name is visible</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Goa</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Airline visible: Air India</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>One Way</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=23/06/2026&amp;from=BLR&amp;to=GOI&amp;intl=n&amp;origin=BLR%20-%20Bengaluru,%20IN&amp;destination=GOI%20-%20Goa,%20IN&amp;sft=&amp;sd=1781331276240&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-06-13T11:44:49</t>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=20/06/2026&amp;from=BOM&amp;to=DEL&amp;intl=n&amp;origin=BOM%20-%20Mumbai,%20IN&amp;destination=DEL%20-%20New%20Delhi,%20IN&amp;sft=&amp;sd=1781341242090&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC001.png</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:30:51</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>TC001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Validate flight price is visible</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Price visible: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=20/06/2026&amp;from=BOM&amp;to=DEL&amp;intl=n&amp;origin=BOM%20-%20Mumbai,%20IN&amp;destination=DEL%20-%20New%20Delhi,%20IN&amp;sft=&amp;sd=1781341242090&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC001.png</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:30:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Validate price format</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Price format valid: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=20/06/2026&amp;from=BOM&amp;to=DEL&amp;intl=n&amp;origin=BOM%20-%20Mumbai,%20IN&amp;destination=DEL%20-%20New%20Delhi,%20IN&amp;sft=&amp;sd=1781341242090&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC001.png</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:30:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Capture screenshot</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Screenshot saved at /Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC001.png</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=20/06/2026&amp;from=BOM&amp;to=DEL&amp;intl=n&amp;origin=BOM%20-%20Mumbai,%20IN&amp;destination=DEL%20-%20New%20Delhi,%20IN&amp;sft=&amp;sd=1781341242090&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC001.png</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:30:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Search flights using Cleartrip flow</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Flight search completed for Bengaluru to Goa</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=23/06/2026&amp;from=BLR&amp;to=GOI&amp;intl=n&amp;origin=BLR%20-%20Bengaluru,%20IN&amp;destination=GOI%20-%20Goa,%20IN&amp;sft=&amp;sd=1781341257807&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC002.png</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Validate airline name is visible</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Airline visible: Air India</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=23/06/2026&amp;from=BLR&amp;to=GOI&amp;intl=n&amp;origin=BLR%20-%20Bengaluru,%20IN&amp;destination=GOI%20-%20Goa,%20IN&amp;sft=&amp;sd=1781341257807&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC002.png</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Validate flight price is visible</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Price visible: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=23/06/2026&amp;from=BLR&amp;to=GOI&amp;intl=n&amp;origin=BLR%20-%20Bengaluru,%20IN&amp;destination=GOI%20-%20Goa,%20IN&amp;sft=&amp;sd=1781341257807&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC002.png</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC002</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Validate price format</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Price format valid: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=23/06/2026&amp;from=BLR&amp;to=GOI&amp;intl=n&amp;origin=BLR%20-%20Bengaluru,%20IN&amp;destination=GOI%20-%20Goa,%20IN&amp;sft=&amp;sd=1781341257807&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC002.png</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Capture screenshot</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Screenshot saved at /Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC002.png</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=23/06/2026&amp;from=BLR&amp;to=GOI&amp;intl=n&amp;origin=BLR%20-%20Bengaluru,%20IN&amp;destination=GOI%20-%20Goa,%20IN&amp;sft=&amp;sd=1781341257807&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC002.png</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>TC003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Search flights using Cleartrip flow</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Flight search completed for Chennai to Hyderabad</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Chennai</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Hyderabad</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>One Way</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>10.47</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=27/06/2026&amp;from=MAA&amp;to=HYD&amp;intl=n&amp;origin=MAA%20-%20Chennai,%20IN&amp;destination=HYD%20-%20Hyderabad,%20IN&amp;sft=&amp;sd=1781331295074&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-06-13T11:45:00</t>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=27/06/2026&amp;from=MAA&amp;to=HYD&amp;intl=n&amp;origin=MAA%20-%20Chennai,%20IN&amp;destination=HYD%20-%20Hyderabad,%20IN&amp;sft=&amp;sd=1781341270221&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC003.png</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC003</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Validate airline name is visible</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Airline visible: Air India</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=27/06/2026&amp;from=MAA&amp;to=HYD&amp;intl=n&amp;origin=MAA%20-%20Chennai,%20IN&amp;destination=HYD%20-%20Hyderabad,%20IN&amp;sft=&amp;sd=1781341270221&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC003.png</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC003</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Validate flight price is visible</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Price visible: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=27/06/2026&amp;from=MAA&amp;to=HYD&amp;intl=n&amp;origin=MAA%20-%20Chennai,%20IN&amp;destination=HYD%20-%20Hyderabad,%20IN&amp;sft=&amp;sd=1781341270221&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC003.png</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC003</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Validate price format</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Price format valid: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=27/06/2026&amp;from=MAA&amp;to=HYD&amp;intl=n&amp;origin=MAA%20-%20Chennai,%20IN&amp;destination=HYD%20-%20Hyderabad,%20IN&amp;sft=&amp;sd=1781341270221&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC003.png</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC003</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Capture screenshot</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Screenshot saved at /Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC003.png</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>One Way</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Verified results at https://www.cleartrip.com/flights/results?adults=1&amp;childs=0&amp;infants=0&amp;class=Economy&amp;depart_date=27/06/2026&amp;from=MAA&amp;to=HYD&amp;intl=n&amp;origin=MAA%20-%20Chennai,%20IN&amp;destination=HYD%20-%20Hyderabad,%20IN&amp;sft=&amp;sd=1781341270221&amp;rnd_one=O&amp;isCfw=false&amp;nonStop=&amp;isFF=false | Airline: Air India | Price: Up to ₹600 off</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>/Users/hannushaik/Downloads/Clear Trip/reports/screenshots/TC003.png</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-06-13T14:31:15</t>
         </is>
       </c>
     </row>

</xml_diff>